<commit_message>
Se Completa el desarrollo de la app
</commit_message>
<xml_diff>
--- a/Gantt_Proyecto_Integrador_IDGS10A_2026_Equipo4_Donaton.xlsx
+++ b/Gantt_Proyecto_Integrador_IDGS10A_2026_Equipo4_Donaton.xlsx
@@ -484,19 +484,19 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -516,23 +516,23 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="9" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="9" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="9" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="9" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="14" fillId="9" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="14" fillId="9" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="10" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="10" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -552,51 +552,51 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="9" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="9" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="12" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="12" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="18" fillId="13" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="18" fillId="13" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="18" fillId="14" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="18" fillId="14" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -604,7 +604,7 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1065,7 +1065,7 @@
       <c r="M8" s="9"/>
       <c r="P8" s="14" t="n">
         <f aca="false">AVERAGE(E5,E6,F7,F8,F9,G10,G11,G12,K13,K14,M15)</f>
-        <v>0.636363636363636</v>
+        <v>0.854545454545455</v>
       </c>
       <c r="Q8" s="14"/>
       <c r="R8" s="14"/>
@@ -1162,7 +1162,7 @@
       <c r="E12" s="9"/>
       <c r="F12" s="9"/>
       <c r="G12" s="17" t="n">
-        <v>0.1</v>
+        <v>1</v>
       </c>
       <c r="H12" s="17"/>
       <c r="I12" s="17"/>
@@ -1191,7 +1191,7 @@
       <c r="I13" s="9"/>
       <c r="J13" s="9"/>
       <c r="K13" s="17" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="L13" s="17"/>
       <c r="M13" s="9"/>
@@ -1216,7 +1216,7 @@
       <c r="I14" s="9"/>
       <c r="J14" s="9"/>
       <c r="K14" s="17" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L14" s="17"/>
       <c r="M14" s="9"/>

</xml_diff>